<commit_message>
Export frozen U-Net matched-crop masks and pixel skeleton root lengths
</commit_message>
<xml_diff>
--- a/roma-results/three-genotypes/UNet-matched-crops-root-length-pixels-20261030/Root_length_matched_crops_pixels.xlsx
+++ b/roma-results/three-genotypes/UNet-matched-crops-root-length-pixels-20261030/Root_length_matched_crops_pixels.xlsx
@@ -692,7 +692,7 @@
       </c>
       <c r="K8" t="inlineStr" s="0">
         <is>
-          <t>未拍摄</t>
+          <t>该期图像缺失</t>
         </is>
       </c>
       <c r="L8" t="inlineStr" s="0">
@@ -746,7 +746,7 @@
       </c>
       <c r="K9" t="inlineStr" s="0">
         <is>
-          <t>未拍摄</t>
+          <t>该期图像缺失</t>
         </is>
       </c>
       <c r="L9" t="inlineStr" s="0">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="J14" t="inlineStr" s="0">
         <is>
-          <t>未拍摄</t>
+          <t>该期图像缺失</t>
         </is>
       </c>
       <c r="K14" t="inlineStr" s="0">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="L16" t="inlineStr" s="0">
         <is>
-          <t>未拍摄</t>
+          <t>该期图像缺失</t>
         </is>
       </c>
     </row>
@@ -1221,7 +1221,7 @@
       </c>
       <c r="J18" t="inlineStr" s="0">
         <is>
-          <t>未拍摄</t>
+          <t>该期图像缺失</t>
         </is>
       </c>
       <c r="K18" t="inlineStr" s="0">
@@ -1280,7 +1280,7 @@
       </c>
       <c r="K19" t="inlineStr" s="0">
         <is>
-          <t>未拍摄</t>
+          <t>该期图像缺失</t>
         </is>
       </c>
       <c r="L19" t="inlineStr" s="0">
@@ -2637,7 +2637,7 @@
       </c>
       <c r="F28" t="inlineStr" s="0">
         <is>
-          <t>未拍摄</t>
+          <t>该期图像缺失</t>
         </is>
       </c>
       <c r="G28" t="inlineStr" s="0">
@@ -2841,7 +2841,7 @@
       </c>
       <c r="F32" t="inlineStr" s="0">
         <is>
-          <t>未拍摄</t>
+          <t>该期图像缺失</t>
         </is>
       </c>
       <c r="G32" t="inlineStr" s="0">
@@ -3765,7 +3765,7 @@
       </c>
       <c r="F51" t="inlineStr" s="0">
         <is>
-          <t>未拍摄</t>
+          <t>该期图像缺失</t>
         </is>
       </c>
       <c r="G51" t="inlineStr" s="0">
@@ -4257,7 +4257,7 @@
       </c>
       <c r="F61" t="inlineStr" s="0">
         <is>
-          <t>未拍摄</t>
+          <t>该期图像缺失</t>
         </is>
       </c>
       <c r="G61" t="inlineStr" s="0">
@@ -4581,7 +4581,7 @@
       </c>
       <c r="F67" t="inlineStr" s="0">
         <is>
-          <t>未拍摄</t>
+          <t>该期图像缺失</t>
         </is>
       </c>
       <c r="G67" t="inlineStr" s="0">
@@ -4833,7 +4833,7 @@
       </c>
       <c r="F72" t="inlineStr" s="0">
         <is>
-          <t>未拍摄</t>
+          <t>该期图像缺失</t>
         </is>
       </c>
       <c r="G72" t="inlineStr" s="0">
@@ -4975,7 +4975,7 @@
       </c>
       <c r="E2" t="inlineStr" s="0">
         <is>
-          <t>未拍摄</t>
+          <t>该期图像缺失</t>
         </is>
       </c>
     </row>
@@ -5000,7 +5000,7 @@
       </c>
       <c r="E3" t="inlineStr" s="0">
         <is>
-          <t>未拍摄</t>
+          <t>该期图像缺失</t>
         </is>
       </c>
     </row>
@@ -5025,7 +5025,7 @@
       </c>
       <c r="E4" t="inlineStr" s="0">
         <is>
-          <t>未拍摄</t>
+          <t>该期图像缺失</t>
         </is>
       </c>
     </row>
@@ -5050,7 +5050,7 @@
       </c>
       <c r="E5" t="inlineStr" s="0">
         <is>
-          <t>未拍摄</t>
+          <t>该期图像缺失</t>
         </is>
       </c>
     </row>
@@ -5150,7 +5150,7 @@
       </c>
       <c r="E9" t="inlineStr" s="0">
         <is>
-          <t>未拍摄</t>
+          <t>该期图像缺失</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E10" t="inlineStr" s="0">
         <is>
-          <t>未拍摄</t>
+          <t>该期图像缺失</t>
         </is>
       </c>
     </row>
@@ -5307,7 +5307,7 @@
       </c>
       <c r="B10" t="inlineStr" s="0">
         <is>
-          <t>NA不代表0。未拍摄与源文件不可用分别列明；每期均值只使用该期实际完成的图像，有效重复数另列。</t>
+          <t>NA不代表0。该期图像缺失与源文件不可用分别列明；每期均值只使用该期实际完成的图像，有效重复数另列。</t>
         </is>
       </c>
     </row>

</xml_diff>